<commit_message>
feat: admin panel at /admin - upload Excel, reset arrivals, remove buttons from main page
</commit_message>
<xml_diff>
--- a/upload/invitados.xlsx
+++ b/upload/invitados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\donal\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A327B754-FA55-4AAB-82DD-438952F3ADD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5C785748-915A-45EA-9906-00DB42052867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7E849B52-6AB6-4F8D-B600-9CC0FFE80195}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="121">
   <si>
     <t>Nombre</t>
   </si>
@@ -151,9 +151,6 @@
     <t>Jorge Acosta (super)</t>
   </si>
   <si>
-    <t>P</t>
-  </si>
-  <si>
     <t>Itis Fernandez y Hermanos</t>
   </si>
   <si>
@@ -172,12 +169,6 @@
     <t>Laura Enriquez</t>
   </si>
   <si>
-    <t>Maestra Edit</t>
-  </si>
-  <si>
-    <t>Rafa y Lety</t>
-  </si>
-  <si>
     <t>Eli y Ana Hdez</t>
   </si>
   <si>
@@ -187,9 +178,6 @@
     <t>Lola y fam.</t>
   </si>
   <si>
-    <t>Profe Valente y Esposa</t>
-  </si>
-  <si>
     <t>Abril Chavarria</t>
   </si>
   <si>
@@ -217,15 +205,15 @@
     <t>Hector Lucero</t>
   </si>
   <si>
-    <t>Maestros - P</t>
-  </si>
-  <si>
     <t>Miguel Armendariz</t>
   </si>
   <si>
     <t>Luki Prieto Jorge</t>
   </si>
   <si>
+    <t>Maestros</t>
+  </si>
+  <si>
     <t>Jorge Chavez y Esp.</t>
   </si>
   <si>
@@ -289,9 +277,6 @@
     <t>Fely Hotel</t>
   </si>
   <si>
-    <t>Palomita</t>
-  </si>
-  <si>
     <t>Marisol</t>
   </si>
   <si>
@@ -382,7 +367,22 @@
     <t>Cintia Ibarra</t>
   </si>
   <si>
-    <t>policia</t>
+    <t>presidencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maestros </t>
+  </si>
+  <si>
+    <t>Policia</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>Rafa y Lety centeno</t>
+  </si>
+  <si>
+    <t>Valente y Esposa</t>
   </si>
 </sst>
 </file>
@@ -1257,7 +1257,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1438,7 +1438,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B22">
         <v>19</v>
@@ -1493,7 +1493,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B23">
         <v>9</v>
@@ -1553,6 +1553,9 @@
       <c r="B28">
         <v>80</v>
       </c>
+      <c r="C28" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -1646,7 +1649,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B38">
         <v>1</v>
@@ -1694,7 +1697,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44">
         <v>6</v>
@@ -1702,7 +1705,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45">
         <v>6</v>
@@ -1710,7 +1713,7 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B46">
         <v>2</v>
@@ -1718,7 +1721,7 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B47">
         <v>4</v>
@@ -1726,7 +1729,7 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B48">
         <v>1</v>
@@ -1734,7 +1737,7 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B49">
         <v>2</v>
@@ -1742,7 +1745,7 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B50">
         <v>2</v>
@@ -1750,18 +1753,18 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>50</v>
+        <v>118</v>
       </c>
       <c r="B51">
         <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>51</v>
+        <v>119</v>
       </c>
       <c r="B52">
         <v>2</v>
@@ -1769,29 +1772,23 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B53">
         <v>2</v>
-      </c>
-      <c r="C53" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B54">
         <v>2</v>
-      </c>
-      <c r="C54" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B55">
         <v>7</v>
@@ -1799,48 +1796,42 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>55</v>
+        <v>120</v>
       </c>
       <c r="B56">
         <v>2</v>
+      </c>
+      <c r="C56" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B57">
         <v>3</v>
-      </c>
-      <c r="C57" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B58">
         <v>2</v>
-      </c>
-      <c r="C58" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B59">
         <v>2</v>
-      </c>
-      <c r="C59" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B60">
         <v>15</v>
@@ -1848,7 +1839,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B61">
         <v>2</v>
@@ -1856,106 +1847,88 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B62">
         <v>3</v>
-      </c>
-      <c r="C62" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B63">
         <v>2</v>
-      </c>
-      <c r="C63" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B64">
         <v>2</v>
-      </c>
-      <c r="C64" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B65">
         <v>2</v>
-      </c>
-      <c r="C65" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B66">
         <v>3</v>
-      </c>
-      <c r="C66" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B67">
         <v>1</v>
       </c>
-      <c r="C67" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B68">
         <v>2</v>
       </c>
       <c r="C68" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B69">
         <v>2</v>
       </c>
       <c r="C69" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B70">
         <v>3</v>
       </c>
       <c r="C70" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B71">
         <v>2</v>
@@ -1963,7 +1936,7 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B72">
         <v>2</v>
@@ -1971,7 +1944,7 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B73">
         <v>2</v>
@@ -1979,7 +1952,7 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B74">
         <v>2</v>
@@ -1987,7 +1960,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B75">
         <v>2</v>
@@ -1995,7 +1968,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B76">
         <v>2</v>
@@ -2003,150 +1976,135 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B77">
         <v>4</v>
       </c>
       <c r="C77" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B78">
         <v>4</v>
       </c>
       <c r="C78" t="s">
-        <v>65</v>
+        <v>116</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B79">
         <v>2</v>
       </c>
       <c r="C79" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B80">
         <v>2</v>
       </c>
       <c r="C80" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B81">
         <v>4</v>
       </c>
       <c r="C81" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B82">
         <v>2</v>
       </c>
       <c r="C82" t="s">
-        <v>65</v>
+        <v>116</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B83">
         <v>4</v>
       </c>
       <c r="C83" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B84">
         <v>1</v>
       </c>
       <c r="C84" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B85">
         <v>2</v>
-      </c>
-      <c r="C85" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B86">
         <v>1</v>
       </c>
-      <c r="C86" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B87">
         <v>1</v>
       </c>
-      <c r="C87" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B88">
         <v>4</v>
       </c>
-      <c r="C88" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B89">
         <v>2</v>
-      </c>
-      <c r="C89" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B90">
         <v>6</v>
@@ -2154,7 +2112,7 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B91">
         <v>4</v>
@@ -2162,7 +2120,7 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B92">
         <v>2</v>
@@ -2170,18 +2128,15 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B93">
         <v>2</v>
-      </c>
-      <c r="C93" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B94">
         <v>2</v>
@@ -2189,7 +2144,7 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B95">
         <v>1</v>
@@ -2197,18 +2152,15 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B96">
         <v>2</v>
-      </c>
-      <c r="C96" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B97">
         <v>2</v>
@@ -2216,51 +2168,39 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B98">
         <v>1</v>
       </c>
-      <c r="C98" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B99">
         <v>2</v>
-      </c>
-      <c r="C99" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B100">
         <v>2</v>
-      </c>
-      <c r="C100" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B101">
         <v>2</v>
-      </c>
-      <c r="C101" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B102">
         <v>2</v>
@@ -2268,18 +2208,15 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B103">
         <v>2</v>
-      </c>
-      <c r="C103" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B104">
         <v>2</v>
@@ -2287,7 +2224,7 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B105">
         <v>2</v>
@@ -2295,7 +2232,7 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B106">
         <v>3</v>
@@ -2303,7 +2240,7 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B107">
         <v>2</v>
@@ -2311,7 +2248,7 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B108">
         <v>4</v>
@@ -2319,7 +2256,7 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B109">
         <v>2</v>
@@ -2327,7 +2264,7 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B110">
         <v>2</v>
@@ -2335,7 +2272,7 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B111">
         <v>2</v>
@@ -2343,13 +2280,13 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B112">
         <v>2</v>
       </c>
       <c r="C112" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: compatibilidad con nuevo Excel (Henandez, Estrada, Especiales, Amigos y trabajo) + endpoint upload + colores
</commit_message>
<xml_diff>
--- a/upload/invitados.xlsx
+++ b/upload/invitados.xlsx
@@ -1,39 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8c30bf0aa213e387/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\donal\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8566262-B9B9-F547-B5DB-DF7922BE5CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{770AF289-F9CC-4A5C-8B98-3F80D4ADF772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7E849B52-6AB6-4F8D-B600-9CC0FFE80195}"/>
   </bookViews>
   <sheets>
     <sheet name="invitados" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="166">
   <si>
     <t>Nombre</t>
   </si>
@@ -41,21 +28,12 @@
     <t>Invitados</t>
   </si>
   <si>
-    <t>Familia Hdez</t>
-  </si>
-  <si>
-    <t>Fam. Estrada</t>
-  </si>
-  <si>
     <t>Angel</t>
   </si>
   <si>
     <t>Victor</t>
   </si>
   <si>
-    <t>DIF</t>
-  </si>
-  <si>
     <t>Cintia</t>
   </si>
   <si>
@@ -122,9 +100,6 @@
     <t>Miguel Armendariz</t>
   </si>
   <si>
-    <t>Maestros</t>
-  </si>
-  <si>
     <t>Tavo Maldonado</t>
   </si>
   <si>
@@ -164,9 +139,6 @@
     <t>Fely Hotel</t>
   </si>
   <si>
-    <t>Profe Fernando</t>
-  </si>
-  <si>
     <t>Cesar Varela</t>
   </si>
   <si>
@@ -200,9 +172,6 @@
     <t>Chela Enriquez</t>
   </si>
   <si>
-    <t>Categori­a/Notas</t>
-  </si>
-  <si>
     <t>Chuy Medina</t>
   </si>
   <si>
@@ -230,24 +199,15 @@
     <t>Cintia Ibarra</t>
   </si>
   <si>
-    <t>presidencia</t>
-  </si>
-  <si>
     <t>Edit</t>
   </si>
   <si>
     <t>Valente y Esposa</t>
   </si>
   <si>
-    <t>Amigos de la familia</t>
-  </si>
-  <si>
     <t>Mario (cuate) y Gladis armendaris y fam.</t>
   </si>
   <si>
-    <t>Familiar lejano</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nancy </t>
   </si>
   <si>
@@ -266,9 +226,6 @@
     <t>Jose Blanco y Lore</t>
   </si>
   <si>
-    <t>Amigos de la familia (Especial)</t>
-  </si>
-  <si>
     <t>Luis Hernandez</t>
   </si>
   <si>
@@ -404,9 +361,6 @@
     <t>Felipe Leon Pacheco</t>
   </si>
   <si>
-    <t>Amigos de la familia (Especial Gobierno)</t>
-  </si>
-  <si>
     <t>LUCIO OLIVAS HERNANDEZ.</t>
   </si>
   <si>
@@ -530,15 +484,9 @@
     <t>Sergio Gonzales y Eposa</t>
   </si>
   <si>
-    <t>Familia</t>
-  </si>
-  <si>
     <t>PRISMA LEDEZMA</t>
   </si>
   <si>
-    <t xml:space="preserve">educación especial </t>
-  </si>
-  <si>
     <t>ZULMA ACOSTA</t>
   </si>
   <si>
@@ -551,13 +499,25 @@
     <t xml:space="preserve">MAGALY VALDEZ </t>
   </si>
   <si>
-    <t>educación especial amigos</t>
-  </si>
-  <si>
     <t>CARLA PRIETO DOMINGUEZ</t>
   </si>
   <si>
     <t>PATY BLANCO</t>
+  </si>
+  <si>
+    <t>Estrada</t>
+  </si>
+  <si>
+    <t>Henandez</t>
+  </si>
+  <si>
+    <t>Especiales</t>
+  </si>
+  <si>
+    <t>Amigos y trabajo</t>
+  </si>
+  <si>
+    <t>Categoria</t>
   </si>
 </sst>
 </file>
@@ -1099,6 +1059,22 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D9764166-3A54-4931-8751-B429079FB14D}" name="Tabla1" displayName="Tabla1" ref="A1:C160" totalsRowShown="0">
+  <autoFilter ref="A1:C160" xr:uid="{D9764166-3A54-4931-8751-B429079FB14D}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{2CEE51E8-81CA-4BE5-AAC2-898B2FE9893D}" name="Nombre"/>
+    <tableColumn id="2" xr3:uid="{709D598B-6935-49BF-A23B-E0C0DD9A8A80}" name="Invitados"/>
+    <tableColumn id="3" xr3:uid="{9B9326D1-F9BC-4EBC-AAEC-CF3B43D6E99E}" name="Categoria"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1418,13 +1394,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9FA23E2-26AC-4798-85B2-68C91D06D323}">
-  <dimension ref="A1:C161"/>
-  <sheetFormatPr defaultColWidth="10.76171875" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C160"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.53515625" customWidth="1"/>
+    <col min="1" max="1" width="30.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1432,1770 +1409,1762 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="B3">
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="B7">
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B8">
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B12">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="B13">
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="B14">
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="B16">
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B17">
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B21">
         <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B22">
         <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B23">
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B24">
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B25">
         <v>6</v>
       </c>
       <c r="C25" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="B26">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B27">
         <v>7</v>
       </c>
       <c r="C27" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B29">
         <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>9</v>
       </c>
       <c r="B31">
         <v>3</v>
       </c>
       <c r="C31" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B33">
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B34">
         <v>3</v>
       </c>
       <c r="C34" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B35">
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B36">
         <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B37">
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B38">
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B39">
         <v>2</v>
       </c>
       <c r="C39" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B40">
         <v>2</v>
       </c>
       <c r="C40" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B41">
         <v>3</v>
       </c>
       <c r="C41" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B42">
         <v>2</v>
       </c>
       <c r="C42" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B43">
         <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B44">
         <v>6</v>
       </c>
       <c r="C44" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B45">
         <v>2</v>
       </c>
       <c r="C45" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B46">
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B47">
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B48">
         <v>4</v>
       </c>
       <c r="C48" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="B49">
         <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>65</v>
+      </c>
+      <c r="B51">
+        <v>2</v>
+      </c>
+      <c r="C51" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>66</v>
       </c>
-      <c r="B50">
-        <v>2</v>
-      </c>
-      <c r="C50" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>74</v>
-      </c>
-      <c r="B51">
-        <v>2</v>
-      </c>
-      <c r="C51" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>75</v>
-      </c>
       <c r="B52">
         <v>2</v>
       </c>
       <c r="C52" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B53">
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B54">
         <v>7</v>
       </c>
       <c r="C54" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B55">
         <v>2</v>
       </c>
       <c r="C55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B56">
         <v>3</v>
       </c>
       <c r="C56" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B57">
         <v>2</v>
       </c>
       <c r="C57" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B58">
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B59">
         <v>15</v>
       </c>
       <c r="C59" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B60">
         <v>2</v>
       </c>
       <c r="C60" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B61">
         <v>3</v>
       </c>
       <c r="C61" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B62">
         <v>2</v>
       </c>
       <c r="C62" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B63">
         <v>2</v>
       </c>
       <c r="C63" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B64">
         <v>2</v>
       </c>
       <c r="C64" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B65">
         <v>3</v>
       </c>
       <c r="C65" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B66">
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="B67">
         <v>2</v>
       </c>
       <c r="C67" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B68">
         <v>2</v>
       </c>
       <c r="C68" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B69">
         <v>3</v>
       </c>
       <c r="C69" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B70">
         <v>2</v>
       </c>
       <c r="C70" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B71">
         <v>2</v>
       </c>
       <c r="C71" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B72">
         <v>2</v>
       </c>
       <c r="C72" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B73">
         <v>2</v>
       </c>
       <c r="C73" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B74">
         <v>2</v>
       </c>
       <c r="C74" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B75">
         <v>2</v>
       </c>
       <c r="C75" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B76">
         <v>4</v>
       </c>
       <c r="C76" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B77">
         <v>4</v>
       </c>
       <c r="C77" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B78">
         <v>2</v>
       </c>
       <c r="C78" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B79">
         <v>2</v>
       </c>
       <c r="C79" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B80">
         <v>4</v>
       </c>
       <c r="C80" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B81">
         <v>2</v>
       </c>
       <c r="C81" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B82">
         <v>4</v>
       </c>
       <c r="C82" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B83">
         <v>1</v>
       </c>
       <c r="C83" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B84">
         <v>2</v>
       </c>
       <c r="C84" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B85">
         <v>1</v>
       </c>
       <c r="C85" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B86">
         <v>1</v>
       </c>
       <c r="C86" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B87">
         <v>4</v>
       </c>
       <c r="C87" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B88">
         <v>2</v>
       </c>
       <c r="C88" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B89">
         <v>2</v>
       </c>
       <c r="C89" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B90">
         <v>2</v>
       </c>
       <c r="C90" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="B91">
         <v>2</v>
       </c>
       <c r="C91" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="B92">
         <v>4</v>
       </c>
       <c r="C92" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>37</v>
+      </c>
+      <c r="B93">
+        <v>2</v>
+      </c>
+      <c r="C93" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>38</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>110</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>39</v>
+      </c>
+      <c r="B96">
+        <v>2</v>
+      </c>
+      <c r="C96" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>40</v>
+      </c>
+      <c r="B97">
+        <v>2</v>
+      </c>
+      <c r="C97" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>111</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>112</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>41</v>
       </c>
-      <c r="B93">
-        <v>2</v>
-      </c>
-      <c r="C93" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+      <c r="B100">
+        <v>2</v>
+      </c>
+      <c r="C100" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>42</v>
       </c>
-      <c r="B94">
-        <v>2</v>
-      </c>
-      <c r="C94" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
+      <c r="B101">
+        <v>2</v>
+      </c>
+      <c r="C101" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>43</v>
+      </c>
+      <c r="B102">
+        <v>2</v>
+      </c>
+      <c r="C102" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>44</v>
+      </c>
+      <c r="B103">
+        <v>2</v>
+      </c>
+      <c r="C103" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>45</v>
+      </c>
+      <c r="B104">
+        <v>2</v>
+      </c>
+      <c r="C104" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>46</v>
+      </c>
+      <c r="B105">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>47</v>
+      </c>
+      <c r="B106">
+        <v>3</v>
+      </c>
+      <c r="C106" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>48</v>
+      </c>
+      <c r="B107">
+        <v>2</v>
+      </c>
+      <c r="C107" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>49</v>
+      </c>
+      <c r="B108">
+        <v>4</v>
+      </c>
+      <c r="C108" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>55</v>
+      </c>
+      <c r="B109">
+        <v>2</v>
+      </c>
+      <c r="C109" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>56</v>
+      </c>
+      <c r="B110">
+        <v>2</v>
+      </c>
+      <c r="C110" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>57</v>
+      </c>
+      <c r="B111">
+        <v>2</v>
+      </c>
+      <c r="C111" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>58</v>
+      </c>
+      <c r="B112">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>148</v>
+      </c>
+      <c r="B113">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>113</v>
+      </c>
+      <c r="B114">
+        <v>2</v>
+      </c>
+      <c r="C114" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>114</v>
+      </c>
+      <c r="B115">
+        <v>2</v>
+      </c>
+      <c r="C115" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>115</v>
+      </c>
+      <c r="B116">
+        <v>2</v>
+      </c>
+      <c r="C116" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>116</v>
+      </c>
+      <c r="B117">
+        <v>2</v>
+      </c>
+      <c r="C117" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>117</v>
+      </c>
+      <c r="B118">
+        <v>2</v>
+      </c>
+      <c r="C118" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>118</v>
+      </c>
+      <c r="B119">
+        <v>2</v>
+      </c>
+      <c r="C119" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>119</v>
+      </c>
+      <c r="B120">
+        <v>2</v>
+      </c>
+      <c r="C120" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
         <v>120</v>
       </c>
-      <c r="B95">
-        <v>2</v>
-      </c>
-      <c r="C95" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>43</v>
-      </c>
-      <c r="B96">
-        <v>1</v>
-      </c>
-      <c r="C96" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>44</v>
-      </c>
-      <c r="B97">
-        <v>2</v>
-      </c>
-      <c r="C97" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>45</v>
-      </c>
-      <c r="B98">
-        <v>2</v>
-      </c>
-      <c r="C98" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
+      <c r="B121">
+        <v>2</v>
+      </c>
+      <c r="C121" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>152</v>
+      </c>
+      <c r="B122">
+        <v>2</v>
+      </c>
+      <c r="C122" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
         <v>121</v>
       </c>
-      <c r="B99">
-        <v>1</v>
-      </c>
-      <c r="C99" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+      <c r="B123">
+        <v>2</v>
+      </c>
+      <c r="C123" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
         <v>122</v>
       </c>
-      <c r="B100">
-        <v>2</v>
-      </c>
-      <c r="C100" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
-        <v>46</v>
-      </c>
-      <c r="B101">
-        <v>2</v>
-      </c>
-      <c r="C101" t="s">
+      <c r="B124">
+        <v>2</v>
+      </c>
+      <c r="C124" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>47</v>
-      </c>
-      <c r="B102">
-        <v>2</v>
-      </c>
-      <c r="C102" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
-        <v>48</v>
-      </c>
-      <c r="B103">
-        <v>2</v>
-      </c>
-      <c r="C103" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
-        <v>49</v>
-      </c>
-      <c r="B104">
-        <v>2</v>
-      </c>
-      <c r="C104" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
-        <v>50</v>
-      </c>
-      <c r="B105">
-        <v>2</v>
-      </c>
-      <c r="C105" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
-        <v>51</v>
-      </c>
-      <c r="B106">
-        <v>2</v>
-      </c>
-      <c r="C106" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
-        <v>52</v>
-      </c>
-      <c r="B107">
+      <c r="B125">
+        <v>2</v>
+      </c>
+      <c r="C125" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>150</v>
+      </c>
+      <c r="B126">
+        <v>2</v>
+      </c>
+      <c r="C126" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>124</v>
+      </c>
+      <c r="B127">
+        <v>2</v>
+      </c>
+      <c r="C127" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>151</v>
+      </c>
+      <c r="B128">
+        <v>2</v>
+      </c>
+      <c r="C128" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>125</v>
+      </c>
+      <c r="B129">
+        <v>2</v>
+      </c>
+      <c r="C129" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>126</v>
+      </c>
+      <c r="B130">
+        <v>2</v>
+      </c>
+      <c r="C130" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>127</v>
+      </c>
+      <c r="B131">
+        <v>2</v>
+      </c>
+      <c r="C131" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>128</v>
+      </c>
+      <c r="B132">
+        <v>2</v>
+      </c>
+      <c r="C132" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>129</v>
+      </c>
+      <c r="B133">
+        <v>2</v>
+      </c>
+      <c r="C133" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>149</v>
+      </c>
+      <c r="B134">
+        <v>2</v>
+      </c>
+      <c r="C134" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>130</v>
+      </c>
+      <c r="B135">
+        <v>2</v>
+      </c>
+      <c r="C135" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>131</v>
+      </c>
+      <c r="B136">
+        <v>2</v>
+      </c>
+      <c r="C136" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>132</v>
+      </c>
+      <c r="B137">
+        <v>2</v>
+      </c>
+      <c r="C137" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>133</v>
+      </c>
+      <c r="B138">
+        <v>2</v>
+      </c>
+      <c r="C138" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>134</v>
+      </c>
+      <c r="B139">
+        <v>2</v>
+      </c>
+      <c r="C139" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>135</v>
+      </c>
+      <c r="B140">
+        <v>2</v>
+      </c>
+      <c r="C140" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>136</v>
+      </c>
+      <c r="B141">
+        <v>2</v>
+      </c>
+      <c r="C141" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>137</v>
+      </c>
+      <c r="B142">
+        <v>2</v>
+      </c>
+      <c r="C142" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>138</v>
+      </c>
+      <c r="B143">
+        <v>2</v>
+      </c>
+      <c r="C143" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>139</v>
+      </c>
+      <c r="B144">
+        <v>2</v>
+      </c>
+      <c r="C144" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>140</v>
+      </c>
+      <c r="B145">
+        <v>2</v>
+      </c>
+      <c r="C145" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>141</v>
+      </c>
+      <c r="B146">
+        <v>2</v>
+      </c>
+      <c r="C146" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>142</v>
+      </c>
+      <c r="B147">
+        <v>2</v>
+      </c>
+      <c r="C147" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>143</v>
+      </c>
+      <c r="B148">
+        <v>2</v>
+      </c>
+      <c r="C148" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>144</v>
+      </c>
+      <c r="B149">
+        <v>2</v>
+      </c>
+      <c r="C149" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>145</v>
+      </c>
+      <c r="B150">
+        <v>2</v>
+      </c>
+      <c r="C150" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>146</v>
+      </c>
+      <c r="B151">
+        <v>2</v>
+      </c>
+      <c r="C151" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>147</v>
+      </c>
+      <c r="B152">
+        <v>2</v>
+      </c>
+      <c r="C152" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>153</v>
+      </c>
+      <c r="B153">
+        <v>2</v>
+      </c>
+      <c r="C153" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>154</v>
+      </c>
+      <c r="B154">
+        <v>2</v>
+      </c>
+      <c r="C154" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>155</v>
+      </c>
+      <c r="B155">
+        <v>2</v>
+      </c>
+      <c r="C155" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>156</v>
+      </c>
+      <c r="B156">
+        <v>2</v>
+      </c>
+      <c r="C156" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>157</v>
+      </c>
+      <c r="B157">
+        <v>2</v>
+      </c>
+      <c r="C157" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>158</v>
+      </c>
+      <c r="B158">
+        <v>4</v>
+      </c>
+      <c r="C158" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>159</v>
+      </c>
+      <c r="B159">
         <v>3</v>
       </c>
-      <c r="C107" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
-        <v>53</v>
-      </c>
-      <c r="B108">
-        <v>2</v>
-      </c>
-      <c r="C108" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
-        <v>54</v>
-      </c>
-      <c r="B109">
-        <v>4</v>
-      </c>
-      <c r="C109" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
-        <v>61</v>
-      </c>
-      <c r="B110">
-        <v>2</v>
-      </c>
-      <c r="C110" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
-        <v>62</v>
-      </c>
-      <c r="B111">
-        <v>2</v>
-      </c>
-      <c r="C111" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
-        <v>63</v>
-      </c>
-      <c r="B112">
-        <v>2</v>
-      </c>
-      <c r="C112" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
-        <v>64</v>
-      </c>
-      <c r="B113">
-        <v>2</v>
-      </c>
-      <c r="C113" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
-        <v>159</v>
-      </c>
-      <c r="B114">
-        <v>2</v>
-      </c>
-      <c r="C114" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>124</v>
-      </c>
-      <c r="B115">
-        <v>2</v>
-      </c>
-      <c r="C115" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
-        <v>125</v>
-      </c>
-      <c r="B116">
-        <v>2</v>
-      </c>
-      <c r="C116" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A117" t="s">
-        <v>126</v>
-      </c>
-      <c r="B117">
-        <v>2</v>
-      </c>
-      <c r="C117" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
-        <v>127</v>
-      </c>
-      <c r="B118">
-        <v>2</v>
-      </c>
-      <c r="C118" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A119" t="s">
-        <v>128</v>
-      </c>
-      <c r="B119">
-        <v>2</v>
-      </c>
-      <c r="C119" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
-        <v>129</v>
-      </c>
-      <c r="B120">
-        <v>2</v>
-      </c>
-      <c r="C120" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A121" t="s">
-        <v>130</v>
-      </c>
-      <c r="B121">
-        <v>2</v>
-      </c>
-      <c r="C121" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
-        <v>131</v>
-      </c>
-      <c r="B122">
-        <v>2</v>
-      </c>
-      <c r="C122" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A123" t="s">
-        <v>163</v>
-      </c>
-      <c r="B123">
-        <v>2</v>
-      </c>
-      <c r="C123" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A124" t="s">
-        <v>132</v>
-      </c>
-      <c r="B124">
-        <v>2</v>
-      </c>
-      <c r="C124" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A125" t="s">
-        <v>133</v>
-      </c>
-      <c r="B125">
-        <v>2</v>
-      </c>
-      <c r="C125" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
-        <v>134</v>
-      </c>
-      <c r="B126">
-        <v>2</v>
-      </c>
-      <c r="C126" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
-        <v>161</v>
-      </c>
-      <c r="B127">
-        <v>2</v>
-      </c>
-      <c r="C127" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
-        <v>135</v>
-      </c>
-      <c r="B128">
-        <v>2</v>
-      </c>
-      <c r="C128" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
-        <v>162</v>
-      </c>
-      <c r="B129">
-        <v>2</v>
-      </c>
-      <c r="C129" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
-        <v>136</v>
-      </c>
-      <c r="B130">
-        <v>2</v>
-      </c>
-      <c r="C130" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A131" t="s">
-        <v>137</v>
-      </c>
-      <c r="B131">
-        <v>2</v>
-      </c>
-      <c r="C131" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
-        <v>138</v>
-      </c>
-      <c r="B132">
-        <v>2</v>
-      </c>
-      <c r="C132" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
-        <v>139</v>
-      </c>
-      <c r="B133">
-        <v>2</v>
-      </c>
-      <c r="C133" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A134" t="s">
-        <v>140</v>
-      </c>
-      <c r="B134">
-        <v>2</v>
-      </c>
-      <c r="C134" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A135" t="s">
+      <c r="C159" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
         <v>160</v>
       </c>
-      <c r="B135">
-        <v>2</v>
-      </c>
-      <c r="C135" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A136" t="s">
-        <v>141</v>
-      </c>
-      <c r="B136">
-        <v>2</v>
-      </c>
-      <c r="C136" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A137" t="s">
-        <v>142</v>
-      </c>
-      <c r="B137">
-        <v>2</v>
-      </c>
-      <c r="C137" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
-        <v>143</v>
-      </c>
-      <c r="B138">
-        <v>2</v>
-      </c>
-      <c r="C138" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A139" t="s">
-        <v>144</v>
-      </c>
-      <c r="B139">
-        <v>2</v>
-      </c>
-      <c r="C139" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
-        <v>145</v>
-      </c>
-      <c r="B140">
-        <v>2</v>
-      </c>
-      <c r="C140" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A141" t="s">
-        <v>146</v>
-      </c>
-      <c r="B141">
-        <v>2</v>
-      </c>
-      <c r="C141" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
-        <v>147</v>
-      </c>
-      <c r="B142">
-        <v>2</v>
-      </c>
-      <c r="C142" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A143" t="s">
-        <v>148</v>
-      </c>
-      <c r="B143">
-        <v>2</v>
-      </c>
-      <c r="C143" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
-        <v>149</v>
-      </c>
-      <c r="B144">
-        <v>2</v>
-      </c>
-      <c r="C144" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A145" t="s">
-        <v>150</v>
-      </c>
-      <c r="B145">
-        <v>2</v>
-      </c>
-      <c r="C145" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A146" t="s">
-        <v>151</v>
-      </c>
-      <c r="B146">
-        <v>2</v>
-      </c>
-      <c r="C146" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A147" t="s">
-        <v>152</v>
-      </c>
-      <c r="B147">
-        <v>2</v>
-      </c>
-      <c r="C147" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A148" t="s">
-        <v>153</v>
-      </c>
-      <c r="B148">
-        <v>2</v>
-      </c>
-      <c r="C148" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A149" t="s">
-        <v>154</v>
-      </c>
-      <c r="B149">
-        <v>2</v>
-      </c>
-      <c r="C149" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A150" t="s">
-        <v>155</v>
-      </c>
-      <c r="B150">
-        <v>2</v>
-      </c>
-      <c r="C150" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A151" t="s">
-        <v>156</v>
-      </c>
-      <c r="B151">
-        <v>2</v>
-      </c>
-      <c r="C151" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A152" t="s">
-        <v>157</v>
-      </c>
-      <c r="B152">
-        <v>2</v>
-      </c>
-      <c r="C152" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A153" t="s">
-        <v>158</v>
-      </c>
-      <c r="B153">
-        <v>2</v>
-      </c>
-      <c r="C153" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A154" t="s">
-        <v>164</v>
-      </c>
-      <c r="B154">
-        <v>2</v>
-      </c>
-      <c r="C154" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A155" t="s">
-        <v>166</v>
-      </c>
-      <c r="B155">
-        <v>2</v>
-      </c>
-      <c r="C155" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A156" t="s">
-        <v>168</v>
-      </c>
-      <c r="B156">
-        <v>2</v>
-      </c>
-      <c r="C156" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A157" t="s">
-        <v>169</v>
-      </c>
-      <c r="B157">
-        <v>2</v>
-      </c>
-      <c r="C157" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A158" t="s">
-        <v>170</v>
-      </c>
-      <c r="B158">
-        <v>2</v>
-      </c>
-      <c r="C158" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A159" t="s">
-        <v>171</v>
-      </c>
-      <c r="B159">
-        <v>4</v>
-      </c>
-      <c r="C159" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A160" t="s">
-        <v>173</v>
-      </c>
       <c r="B160">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C160" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A161" t="s">
-        <v>174</v>
-      </c>
-      <c r="B161">
-        <v>2</v>
-      </c>
-      <c r="C161" t="s">
-        <v>68</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>